<commit_message>
Add changes required for PeerJS review
</commit_message>
<xml_diff>
--- a/analysis/S1_Table.xlsx
+++ b/analysis/S1_Table.xlsx
@@ -663,11 +663,7 @@
           <t>Claude Opus 4.6</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="D5" s="3" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr">
         <is>
           <t>GPT-OSS 120B</t>
@@ -703,11 +699,7 @@
           <t>Claude Sonnet 4.6</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="D6" s="3" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr">
         <is>
           <t>GPT-OSS 120B</t>

</xml_diff>